<commit_message>
Add Instagram handles to NYC and LA brand scouting spreadsheets
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/adminfiles/smthg_California_LA_scouting_base_v1.xlsx
+++ b/adminfiles/smthg_California_LA_scouting_base_v1.xlsx
@@ -72,7 +72,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -85,6 +85,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -451,7 +452,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P21"/>
+  <dimension ref="A1:Q21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -470,6 +471,7 @@
     <col width="58" customWidth="1" min="14" max="14"/>
     <col width="38" customWidth="1" min="15" max="15"/>
     <col width="50" customWidth="1" min="16" max="16"/>
+    <col width="38" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1" ht="38" customHeight="1">
@@ -553,6 +555,11 @@
           <t>Primary source</t>
         </is>
       </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -633,6 +640,11 @@
           <t>https://www.vogue.com/fashion-shows/designer/erl</t>
         </is>
       </c>
+      <c r="Q2" s="6" t="inlineStr">
+        <is>
+          <t>@erl</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -713,6 +725,11 @@
           <t>https://nahmias.com/pages/about</t>
         </is>
       </c>
+      <c r="Q3" s="6" t="inlineStr">
+        <is>
+          <t>@nahmias__</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -793,6 +810,11 @@
           <t>https://www.vogue.com/fashion-shows/no-sesso</t>
         </is>
       </c>
+      <c r="Q4" s="6" t="inlineStr">
+        <is>
+          <t>@nosessola</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -873,6 +895,11 @@
           <t>https://www.businessoffashion.com/articles/entrepreneurship/how-raisefashions-emerging-designers-build-brands-informed-by-heritage/</t>
         </is>
       </c>
+      <c r="Q5" s="6" t="inlineStr">
+        <is>
+          <t>@houseofaama</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -953,6 +980,11 @@
           <t>https://onlineceramics.shop/</t>
         </is>
       </c>
+      <c r="Q6" s="6" t="inlineStr">
+        <is>
+          <t>@onlineceramics</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -1033,6 +1065,11 @@
           <t>https://www.fashionbrandcompany.com/pages/about</t>
         </is>
       </c>
+      <c r="Q7" s="6" t="inlineStr">
+        <is>
+          <t>@fashionbrandcompany</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -1113,6 +1150,11 @@
           <t>https://slamjam.com/collections/pleasures</t>
         </is>
       </c>
+      <c r="Q8" s="6" t="inlineStr">
+        <is>
+          <t>@pleasures</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1193,6 +1235,11 @@
           <t>https://magazine.032c.com/magazine/the-architecture-of-expansion-with-dylan-richards-diaz-of-entire-studios</t>
         </is>
       </c>
+      <c r="Q9" s="6" t="inlineStr">
+        <is>
+          <t>@entire_studios</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1265,12 +1312,17 @@
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>https://geel.us/</t>
         </is>
       </c>
       <c r="P10" s="3" t="inlineStr">
         <is>
           <t>https://www.whowhatwear.com/fashion/shopping/brand-discovery-2025</t>
+        </is>
+      </c>
+      <c r="Q10" s="2" t="inlineStr">
+        <is>
+          <t>@geel.us</t>
         </is>
       </c>
     </row>
@@ -1353,6 +1405,11 @@
           <t>https://www.vogue.com/fashion-shows/miaou</t>
         </is>
       </c>
+      <c r="Q11" s="6" t="inlineStr">
+        <is>
+          <t>@miaou</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1433,6 +1490,11 @@
           <t>https://www.kindredblack.com/blogs/journal/kindred-black-x-j-hannah</t>
         </is>
       </c>
+      <c r="Q12" s="6" t="inlineStr">
+        <is>
+          <t>@j.hannah</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1513,6 +1575,11 @@
           <t>https://www.ssense.com/en-us/women/designers/emme-parsons</t>
         </is>
       </c>
+      <c r="Q13" s="6" t="inlineStr">
+        <is>
+          <t>@emmeparsons</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1593,6 +1660,11 @@
           <t>https://fashionista.com/2025/02/new-arrivals-spring-2025-best-brands-clothing-accessories-drops</t>
         </is>
       </c>
+      <c r="Q14" s="6" t="inlineStr">
+        <is>
+          <t>@shopdoen</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1673,6 +1745,11 @@
           <t>https://www.whowhatwear.com/fashion/shopping/tops-dresses-summer-2026</t>
         </is>
       </c>
+      <c r="Q15" s="6" t="inlineStr">
+        <is>
+          <t>@ciao__lucia</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1753,6 +1830,11 @@
           <t>https://www.cosimo.shop/brands/rue-sophie</t>
         </is>
       </c>
+      <c r="Q16" s="6" t="inlineStr">
+        <is>
+          <t>@rue__sophie</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1833,6 +1915,11 @@
           <t>https://www.discobrands.co/blogs/20-brands-like-la-streetwear-brands</t>
         </is>
       </c>
+      <c r="Q17" s="6" t="inlineStr">
+        <is>
+          <t>@bornxraised</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1913,6 +2000,11 @@
           <t>https://www.vogue.com/fashion-shows/designer/one-of-these-days</t>
         </is>
       </c>
+      <c r="Q18" s="6" t="inlineStr">
+        <is>
+          <t>@oneofthesedaysco</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1993,6 +2085,11 @@
           <t>https://niathebrand.com/pages/about-us</t>
         </is>
       </c>
+      <c r="Q19" s="6" t="inlineStr">
+        <is>
+          <t>@niathebrand</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -2073,6 +2170,11 @@
           <t>https://nahmias.com/pages/about</t>
         </is>
       </c>
+      <c r="Q20" s="6" t="inlineStr">
+        <is>
+          <t>@nahmias__</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -2151,6 +2253,11 @@
       <c r="P21" s="3" t="inlineStr">
         <is>
           <t>https://www.vogue.com/fashion-shows/designer/amiri</t>
+        </is>
+      </c>
+      <c r="Q21" s="6" t="inlineStr">
+        <is>
+          <t>@amiri</t>
         </is>
       </c>
     </row>

</xml_diff>